<commit_message>
Fix Salazar/Abril ranking issues and update admin UI
</commit_message>
<xml_diff>
--- a/dist/docs/Ranking Catalán 2026.xlsx
+++ b/dist/docs/Ranking Catalán 2026.xlsx
@@ -60,8 +60,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Etapa 1 Masculino'!$B$2:$F$22</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="33" hidden="1">'Etapa 4 Senior'!$B$2:$G$7</definedName>
   </definedNames>
-  <calcPr calcId="191029" calcCompleted="0" forceFullCalc="1"/>
-  <fileRecoveryPr repairLoad="1"/>
+  <calcPr calcId="191029" forceFullCalc="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -642,6 +641,7 @@
     <font>
       <sz val="8"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="9">

</xml_diff>